<commit_message>
Fix depletion_rate/cohort_index/promo_diff common-support bug (was fabricating large moves across scope changes); ship RC collector disabled pending region-data fix; promo reference + diff with offer-level detail
</commit_message>
<xml_diff>
--- a/reports/2026-09-16__daily-marker.xlsx
+++ b/reports/2026-09-16__daily-marker.xlsx
@@ -14,14 +14,15 @@
     <sheet name="Cohort index" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Depletion" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Promo diff" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Promo reference" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$41:$D$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$42:$D$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Availability'!$A$15:$P$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Peer gap'!$A$17:$L$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Earnings window'!$A$11:$I$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cohort index'!$A$17:$S$64</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Promo diff'!$A$11:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Promo reference'!$A$14:$Q$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -612,7 +613,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-16T06:51:47+00:00</t>
+          <t>2026-09-16T16:45:49+00:00</t>
         </is>
       </c>
     </row>
@@ -773,7 +774,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>SINCE INCEPTION = ONE DAY. The panel holds a single collection date (2026-09-16)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -829,99 +830,109 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>no rows</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Which offers widened, narrowed, appeared or were withdrawn between dates, by reach on cabins seen both times.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Promo reference</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>promo-reference</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>reference (every date in the tier)</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>15</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Promo churn per line across collection dates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>The decoder ring: every offer observed, in the vendor's own words, with its reach and scope. Read the Promo diff against this rather than against a hash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Region coverage on this basis</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Every region the config asks for, including those that returned nothing. A region with 0 rows is absent from every sheet; without this table that is indistinguishable from a region nobody requested.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>region</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>observations</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>sailings</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>lines</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>package_rows</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Caribbean</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>431</v>
-      </c>
-      <c r="C31" t="n">
-        <v>90</v>
-      </c>
-      <c r="D31" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Southern Europe</t>
+          <t>Caribbean</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>80</v>
+        <v>431</v>
       </c>
       <c r="C32" t="n">
-        <v>14</v>
+        <v>90</v>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
@@ -931,14 +942,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Northern Europe</t>
+          <t>Southern Europe</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D33" t="n">
         <v>1</v>
@@ -951,17 +962,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Northern Europe</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="C34" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
@@ -971,103 +982,123 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Alaska</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>no rows on this basis -- absent from every sheet</t>
-        </is>
-      </c>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Alaska</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>no rows on this basis -- absent from every sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>Transatlantic</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>0</v>
-      </c>
-      <c r="C36" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" t="inlineStr">
+      <c r="B37" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="inlineStr">
         <is>
           <t>no rows on this basis -- absent from every sheet</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Scope comparability between collection dates</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Whether each pair of adjacent collection dates sampled the same population. Where `comparable` is NO, the collector itself changed, and every slope or index spanning that pair is measuring the change to the collector as well as the market.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>from_date</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>to_date</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>comparable</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>why_not</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>fewer than two collection dates in this tier</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A41:D42"/>
+  <autoFilter ref="A42:D43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8101,37 +8132,158 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Promo diff</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Which offers widened, narrowed, appeared or were withdrawn between dates, by reach on cabins seen both times.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Time scope: all scrape dates in the tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>[daily-marker] sail 2026-10-01..2026-12-31 | regions: Bermuda, Caribbean, Northern Europe, Southern Europe | observed 2026-09-16 | 562 obs / 113 sailings | granularity: category</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>! daily-marker is the Oct-Dec 2026 near-term cohort, and its region mix is set by seasonal deployment, not by sampling choice. Measured from the near-term universe on 2026-09-15: Caribbean 104 eligible itineraries (85 NCL / 19 Carnival); Southern Europe 15, ALL NCL, all departing October-early November, 0 in December and 0 on Carnival; Alaska 0. So cross-line work in this tier is Caribbean-only, and its Southern Europe rows are a single-line October series that dies when the Mediterranean season ends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>! PEER-COMPARABLE REGIONS in this basis: Bermuda, Caribbean. Single-line only (no peer rows, so no cross-line claim can rest on them): Northern Europe (Norwegian Cruise Line), Southern Europe (Norwegian Cruise Line).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>! ONE-SIDED: Carnival Cruise Line, Royal Caribbean International publish no offer detail, so this table can only describe NCLH's promotional behaviour. It cannot support 'NCLH is discounting harder than the peer' -- the peer's discounting is not observable here at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>! NO CHURN OBSERVABLE: no group has cabins carrying offer data on two collection dates in this scope, so nothing can have changed yet. More than one collection date is not the same as two readings of the same inventory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>- COMMON SUPPORT: shares are the fraction of cabins observed on BOTH dates that carried the offer. Sailings entering the book cannot move them, so a widened collection scope cannot read as a promo change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>- naive_* is share of everything each date returned; mix_effect_pp is how many points of the naive move are composition rather than offer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>- Reach, not count: an offer on one ship and an offer fleet-wide are both 'one promo', and the difference is the whole signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>- status: NEW / WITHDRAWN are appearance and disappearance on matched cabins; widened and narrowed are reach moves beyond 2 points.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>- A promotion that deepens without widening does not show here: this measures reach, not discount depth. Depth is in the fare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>(no rows)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="46" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Promo diff</t>
+          <t>Promo reference</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Promo churn per line across collection dates.</t>
+          <t>The decoder ring: every offer observed, in the vendor's own words, with its reach and scope. Read the Promo diff against this rather than against a hash.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Time scope: all scrape dates in the tier.</t>
+          <t>Time scope: reference (every date in the tier).</t>
         </is>
       </c>
     </row>
@@ -8157,115 +8309,1295 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>- promo_hash is a stable hash of the sorted (code, title, inclusion) triples, so churn means the offer really changed, not that the payload was reordered.</t>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>! NOT ALL LINES PUBLISH OFFERS: Carnival Cruise Line, Royal Caribbean International expose no promo detail at all, so their absence from this table is a gap in the source, not evidence that they are not discounting. Any cross-line read on promotion intensity is one-sided.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>- Bodies are in the `promos` table; Store.promo_text(hash) resolves one.</t>
+          <t>- One row per (line, offer code). A promo_hash is a bundle of offers, so one bundle contributes to several rows; `bundles` counts how many distinct bundles carried this offer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>- share_of_line_cells is out of ALL that line's cells in scope, priced or not, so it reads as reach across the book.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>- `inclusion` = Mandatory means the vendor applies it automatically; it is a headline fare condition, not an opt-in the shopper chose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>- Text is the vendor's own, verbatim from the archived payload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>line</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>scrape_date</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>inclusion</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>offer_type</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>featured</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>cells</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>promo_share</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>distinct_promos</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>new_promos</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>dropped_promos</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Carnival Cruise Line</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>256</v>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>line does not expose promo detail</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>share_of_line_cells</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>regions</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>cabin_categories</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>n_ships</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>bundles</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>first_scrape</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>last_scrape</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>sail_from</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>sail_to</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Norwegian Cruise Line</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>306</v>
-      </c>
-      <c r="D13" s="7" t="n">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>50-off-all-cruises-offer</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>50% Off All Cruises</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>auto-included-offer</t>
+        </is>
+      </c>
+      <c r="F15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>248</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>0.8105</v>
       </c>
-      <c r="E13" t="n">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean, Northern Europe, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>11</v>
+      </c>
+      <c r="L15" t="n">
         <v>10</v>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>ok</t>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Save big with 50% off cruise fares for all guests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>travel-protection-norwegiancare</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Travel Protection | NorwegianCare</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>travel-protection-offer</t>
+        </is>
+      </c>
+      <c r="F16" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>248</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>0.8105</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean, Northern Europe, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>11</v>
+      </c>
+      <c r="L16" t="n">
+        <v>10</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Travel
+Protection can help with unforeseen circumstances and get your trip covered
+from shore to ship.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>travel-protection-essentials</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Travel Protection | Essentials</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>travel-protection-offer</t>
+        </is>
+      </c>
+      <c r="F17" t="b">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>248</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>0.8105</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean, Northern Europe, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>11</v>
+      </c>
+      <c r="L17" t="n">
+        <v>10</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Travel Protection | Essentials</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>prepaid-service-charges</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Prepaid Service Charges</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>prepaid-service-charge-offer</t>
+        </is>
+      </c>
+      <c r="F18" t="b">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>248</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>0.8105</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean, Northern Europe, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>11</v>
+      </c>
+      <c r="L18" t="n">
+        <v>10</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Prepaying gratuities can provide peace of mind for a smoother cruise experience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>50-pct-Off-All-Cruises-Offer</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>50% Off All Cruises</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>stateroom-offer</t>
+        </is>
+      </c>
+      <c r="F19" t="b">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>248</v>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>0.8105</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean, Northern Europe, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>11</v>
+      </c>
+      <c r="L19" t="n">
+        <v>10</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Save big with 50% off cruise fares for all guests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>unlimited-open-bar-offer</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Removable</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>beverage-package-offer</t>
+        </is>
+      </c>
+      <c r="F20" t="b">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>248</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>0.8105</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean, Northern Europe, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>11</v>
+      </c>
+      <c r="L20" t="n">
+        <v>10</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Enjoy the best beverage package at sea! Indulge in unlimited
+premium spirits such as Grey Goose, Casamigos, Woodford Reserve and more, plus
+cocktails, wine, beer, soft drinks and juice — all included. Simply pay the
+package gratuities in advance, and the drinks are on us. With drinks on board
+averaging $15 each, there’s no better value.&lt;/p&gt;&lt;p&gt;Gratuities are $32 per person, per day for 2–5 night
+sailings and $28.50 per person, per day for sailings of 6 nights or more. This
+is reflected in the total price shown above and in the guest breakdown.&lt;br&gt;&lt;/p&gt;&lt;p&gt;The package applies to all guests in the stateroom aged 21+.
+Guests 1 or 2 under age 21 will instead receive juice and unlimited fountain
+soda for $12.50 per person per day. Guests 3–8 under 21 will not receive a
+beverage package but may purchase one separately.&lt;/p&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>specialty-dining-offer</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Dining</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Removable</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>dining-offer</t>
+        </is>
+      </c>
+      <c r="F21" t="b">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>248</v>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>0.8105</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean, Northern Europe, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>11</v>
+      </c>
+      <c r="L21" t="n">
+        <v>10</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Savor amazing multi-course meals at our award-winning Specialty Restaurants, such as Cagney’s Steakhouse or Le Bistro. Enjoy elevated dining experiences featuring globally inspired cuisine and exceptional service — all included. Simply pre-pay the package gratuities in advance, and the dining experience is on us. With an average of $60 per meal onboard, this value can’t be beat. &lt;br&gt;  &lt;br&gt;   The package applies to all guests on the reservation.  Guests under age 13 dine for free when ordering from the kids’ menu. If they choose to order from the specialty dining menu, a $20 cover charge will apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>free-wifi-offer</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Wi-Fi Package</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>wifi-package-offer</t>
+        </is>
+      </c>
+      <c r="F22" t="b">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>248</v>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>0.8105</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean, Northern Europe, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>11</v>
+      </c>
+      <c r="L22" t="n">
+        <v>10</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Stay connected throughout your cruise with 150 minutes of hi-speed Wi-Fi per person included. Offer applies to all guests in the stateroom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>excursion-credits-offer</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Excursion Credits</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>shorex-offer</t>
+        </is>
+      </c>
+      <c r="F23" t="b">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>248</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>0.8105</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean, Northern Europe, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>11</v>
+      </c>
+      <c r="L23" t="n">
+        <v>10</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Receive a $50 credit toward every shore excursion. Offer applies to the first guest on the reservation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>specialty-dining-offer-7-8-nights</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Dining</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Removable</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>dining-offer</t>
+        </is>
+      </c>
+      <c r="F24" t="b">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>209</v>
+      </c>
+      <c r="H24" s="7" t="n">
+        <v>0.6830000000000001</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>8</v>
+      </c>
+      <c r="L24" t="n">
+        <v>5</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Savor 3 amazing multi-course meals at our award-winning Specialty Restaurants, such as Cagney’s Steakhouse or Le Bistro. Enjoy elevated dining experiences featuring globally inspired cuisine and exceptional service — all included. Simply pre-pay the package gratuities in advance, and the dining experience is on us. With an average of $60 per meal onboard, this value can’t be beat. &lt;br&gt;  &lt;br&gt;  The package applies to all guests on the reservation.  Guests under age 13 dine for free when ordering from the kids’ menu. If they choose to order from the specialty dining menu, a $20 cover charge will apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Kids-Sail-Free-Offer</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Kids Sail Free</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>auto-included-offer</t>
+        </is>
+      </c>
+      <c r="F25" t="b">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>152</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>0.4967</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>9</v>
+      </c>
+      <c r="L25" t="n">
+        <v>5</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>2026-12-13</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>3rd &amp; 4th guests in the same stateroom pay only taxes, and fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Past-Guest-Offer</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Past Guest Offer</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>auto-included-offer</t>
+        </is>
+      </c>
+      <c r="F26" t="b">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>37</v>
+      </c>
+      <c r="H26" s="7" t="n">
+        <v>0.1209</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>6</v>
+      </c>
+      <c r="L26" t="n">
+        <v>4</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>2026-12-13</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Extra Latitudes Point</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>specialty-dining-offer-9-nights</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Dining</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Removable</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>dining-offer</t>
+        </is>
+      </c>
+      <c r="F27" t="b">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>23</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>0.0752</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Northern Europe, Southern Europe</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>3</v>
+      </c>
+      <c r="L27" t="n">
+        <v>2</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Savor 4 amazing multi-course meals at our award-winning Specialty Restaurants, such as Cagney’s Steakhouse or Le Bistro. Enjoy elevated dining experiences featuring globally inspired cuisine and exceptional service — all included. Simply pre-pay the package gratuities in advance, and the dining experience is on us. With an average of $60 per meal onboard, this value can’t be beat.&lt;br&gt;   &lt;br&gt;    The package applies to all guests on the reservation.  Guests under age 13 dine for free when ordering from the kids’ menu. If they choose to order from the specialty dining menu, a $20 cover charge will apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>specialty-dining-offer-5-6-nights</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Dining</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Removable</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>dining-offer</t>
+        </is>
+      </c>
+      <c r="F28" t="b">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>16</v>
+      </c>
+      <c r="H28" s="7" t="n">
+        <v>0.0523</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Bermuda, Caribbean</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>2</v>
+      </c>
+      <c r="L28" t="n">
+        <v>3</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>2026-11-11</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Savor 2 amazing multi-course meals at our award-winning Specialty Restaurants, such as Cagney’s Steakhouse or Le Bistro. Enjoy elevated dining experiences featuring globally inspired cuisine and exceptional service — all included. Simply pre-pay the package gratuities in advance, and the dining experience is on us. With an average of $60 per meal onboard, this value can’t be beat.&lt;br&gt; &lt;br&gt; The package applies to all guests on the reservation.  Guests under age 13 dine for free when ordering from the kids’ menu. If they choose to order from the specialty dining menu, a $20 cover charge will apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Norwegian Cruise Line</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>latitudes-rewards-members-cruise</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Latitudes Annual Member Cruise</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>auto-included-offer</t>
+        </is>
+      </c>
+      <c r="F29" t="b">
+        <v>1</v>
+      </c>
+      <c r="G29" t="n">
+        <v>6</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <v>0.0196</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Caribbean</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>balcony, inside, oceanview, suite</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>1</v>
+      </c>
+      <c r="L29" t="n">
+        <v>1</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>2026-12-06</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>2026-12-06</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Latitudes Member Cruise</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A11:H13"/>
+  <autoFilter ref="A14:Q29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>